<commit_message>
Refactor Strava refresh and static publishing
</commit_message>
<xml_diff>
--- a/data/teams.xlsx
+++ b/data/teams.xlsx
@@ -413,54 +413,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>team_name</t>
+          <t>Team 1</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>members</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>distance</t>
+          <t>Team 2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Team 1</t>
+          <t>TheoD.</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TheoD.,LucasH.,NoahB.</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>22785.1</v>
+          <t>AlexL.</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Team 2</t>
+          <t>LucasH.</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AlexL.,StanislasD.,RaphC.</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>98851.90000000001</v>
+          <t>StanislasD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NoahB.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RaphC.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajout des équipes pour la course
</commit_message>
<xml_diff>
--- a/data/teams.xlsx
+++ b/data/teams.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duthilt2\Desktop\ESIEE\Club-Running\running_team_vs\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\duthilt2\Desktop\ESIEE\Club-Running\running_team_vs_temp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4FF9B09-56F4-4C60-9CEB-4E9A992E618A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F53E033-5467-4673-81CE-09CF808CB7F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,18 +20,174 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Team 1</t>
-  </si>
-  <si>
-    <t>Team 2</t>
-  </si>
-  <si>
-    <t>TheoD.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+  <si>
+    <t>Brazilian Baddies Lover</t>
+  </si>
+  <si>
+    <t>Honorable</t>
+  </si>
+  <si>
+    <t>NoahB.</t>
+  </si>
+  <si>
+    <t>Les poules pondeuses</t>
+  </si>
+  <si>
+    <t>YaelS.</t>
+  </si>
+  <si>
+    <t>LeonR.</t>
+  </si>
+  <si>
+    <t>VincentP.</t>
+  </si>
+  <si>
+    <t>ClementL.</t>
+  </si>
+  <si>
+    <t>MAMA l'équipe</t>
+  </si>
+  <si>
+    <t>MathisG.</t>
+  </si>
+  <si>
+    <t>Mederic</t>
+  </si>
+  <si>
+    <t>AntoL.</t>
+  </si>
+  <si>
+    <t>AgatheM.</t>
+  </si>
+  <si>
+    <t>Les Loulous</t>
+  </si>
+  <si>
+    <t>CelestinL.</t>
+  </si>
+  <si>
+    <t>ThibaultL.</t>
+  </si>
+  <si>
+    <t>LucasL.</t>
+  </si>
+  <si>
+    <t>EnzoL.</t>
+  </si>
+  <si>
+    <t>Esiee en sueur</t>
+  </si>
+  <si>
+    <t>EthanS.</t>
+  </si>
+  <si>
+    <t>RomaneJ.</t>
+  </si>
+  <si>
+    <t>ClémentG.</t>
+  </si>
+  <si>
+    <t>BenB.</t>
+  </si>
+  <si>
+    <t>67 kilometers</t>
+  </si>
+  <si>
+    <t>EstebanB.</t>
+  </si>
+  <si>
+    <t>MatheoD.</t>
+  </si>
+  <si>
+    <t>ValentinC.</t>
+  </si>
+  <si>
+    <t>UsmanS.</t>
+  </si>
+  <si>
+    <t>Les asiats</t>
+  </si>
+  <si>
+    <t>LyneV.</t>
+  </si>
+  <si>
+    <t>CamilleK.</t>
+  </si>
+  <si>
+    <t>Les Teambrés</t>
+  </si>
+  <si>
+    <t>ArsèneD.</t>
+  </si>
+  <si>
+    <t>ThomasL.</t>
+  </si>
+  <si>
+    <t>PabloC.</t>
+  </si>
+  <si>
+    <t>RomainP.</t>
+  </si>
+  <si>
+    <t>Burger</t>
   </si>
   <si>
     <t>SelmaR.</t>
+  </si>
+  <si>
+    <t>BaptisteM.</t>
+  </si>
+  <si>
+    <t>CamilleF.</t>
+  </si>
+  <si>
+    <t>SachaB.</t>
+  </si>
+  <si>
+    <t>Akatsuki</t>
+  </si>
+  <si>
+    <t>SteveD.</t>
+  </si>
+  <si>
+    <t>GeorgeM.</t>
+  </si>
+  <si>
+    <t>LucieD.</t>
+  </si>
+  <si>
+    <t>NolanP.</t>
+  </si>
+  <si>
+    <t>Lukético</t>
+  </si>
+  <si>
+    <t>TimothéeP.</t>
+  </si>
+  <si>
+    <t>LucienP.</t>
+  </si>
+  <si>
+    <t>KevinP.</t>
+  </si>
+  <si>
+    <t>CorentinP.</t>
+  </si>
+  <si>
+    <t>Les mixés</t>
+  </si>
+  <si>
+    <t>ThéoD.</t>
+  </si>
+  <si>
+    <t>KévinB.</t>
+  </si>
+  <si>
+    <t>CorentinB.</t>
+  </si>
+  <si>
+    <t>sg.</t>
   </si>
 </sst>
 </file>
@@ -371,23 +527,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K2" t="s">
+        <v>47</v>
+      </c>
+      <c r="L2" t="s">
+        <v>52</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>